<commit_message>
Fix input files for hydroExample
Switch to newest InOutModule
Remove calc_no_spinup.py
Rename hydro_old_formulation.py
</commit_message>
<xml_diff>
--- a/data/hydroExample/Global_Scenarios.xlsx
+++ b/data/hydroExample/Global_Scenarios.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\FelixAuer\Git\LEGO-Pyomo2\data\hydroExample\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37756F64-B6C4-4F08-AA25-28B2B4C90B97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7D5B7CB-4467-47EB-A02D-D1F83E1374A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34230" yWindow="-21705" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-4170" yWindow="-21720" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Scenarios" sheetId="1" r:id="rId1"/>
@@ -222,26 +222,31 @@
       <b/>
       <sz val="11"/>
       <name val="Aptos"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="11"/>
       <name val="Aptos"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
       <name val="Aptos"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="18"/>
       <color rgb="FFFFFFFF"/>
       <name val="Aptos"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Aptos"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="8"/>
@@ -743,7 +748,9 @@
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="10"/>
+      <c r="A8" s="10" t="s">
+        <v>23</v>
+      </c>
       <c r="B8" s="11"/>
       <c r="C8" s="12" t="s">
         <v>24</v>
@@ -771,9 +778,7 @@
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="10" t="s">
-        <v>23</v>
-      </c>
+      <c r="A10" s="10"/>
       <c r="B10" s="11"/>
       <c r="C10" s="12" t="s">
         <v>26</v>

</xml_diff>